<commit_message>
Patiëntvriendelijke teksten + fix stadsnamen + Google Maps links
</commit_message>
<xml_diff>
--- a/data/aandoeningen.xlsx
+++ b/data/aandoeningen.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Chronische ontstekingsziekte van de luchtwegen met aanvallen van kortademigheid, piepende ademhaling en hoest.</t>
+          <t>Bij astma zijn uw luchtwegen chronisch ontstoken en extra gevoelig. Dat kan leiden tot aanvallen van kortademigheid, piepende ademhaling en hoest. Met de juiste medicatie en opvolging houdt u astma goed onder controle.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -541,7 +541,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Overgevoeligheidsreacties op allergenen zoals pollen, huisstofmijt of dieren. Diagnose via huidtesten, behandeling via antihistaminica of immunotherapie.</t>
+          <t>Uw lichaam reageert overdreven op stoffen zoals pollen, huisstofmijt of dierenharen. Via huidtesten of bloedonderzoek sporen wij het allergeen op. De behandeling bestaat uit medicatie of desensibilisatie (immunotherapie).</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -571,7 +571,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Chronisch obstructief longlijden door langdurige luchtwegontsteking, meist door roken. Behandeling via bronchusverwijders, revalidatie en rookstop.</t>
+          <t>COPD is een chronische longziekte waarbij uw luchtwegen vernauwd raken, meestal door jarenlang roken. U ervaart toenemende kortademigheid, hoest en slijm. Rookstop, medicatie en longrevalidatie vertragen de achteruitgang aanzienlijk.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Infectie van het longweefsel door bacteriën, virussen of schimmels.</t>
+          <t>Een longontsteking is een infectie van het longweefsel, veroorzaakt door bacteriën, virussen of schimmels. Typische klachten zijn koorts, hoest, kortademigheid en vermoeidheid. De meeste longontstekingen genezen goed met de juiste behandeling.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Spontane of traumatische longcollaps waarbij lucht in de pleurale ruimte komt.</t>
+          <t>Bij een klaplong ontsnapt er lucht uit de long naar de borstholte, waardoor de long (deels) samenvalt. Dit kan spontaan optreden of na een trauma. U voelt plotse stekende pijn op de borst en kortademigheid.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bloedklonter in de longslagaderen, vaak afkomstig van diepe veneuze trombose.</t>
+          <t>Een longembolie ontstaat wanneer een bloedklonter een bloedvat in de longen blokkeert, meestal afkomstig uit een beenader. Klachten zijn plotse kortademigheid, pijn op de borst en soms bloed ophoesten. Snelle diagnose en bloedverdunners zijn essentieel.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Kwaadaardige tumor van het longweefsel. Multidisciplinaire aanpak via wekelijks MOC-overleg.</t>
+          <t>Longkanker is een kwaadaardige tumor in het longweefsel. Klachten zoals aanhoudende hoest, bloed ophoesten of gewichtsverlies treden vaak pas laat op. Bij AZORG bespreken we elke patiënt wekelijks in een multidisciplinair overleg (MOC) voor de best mogelijke behandeling.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Granulomateuze ziekte die de longen, klieren en andere organen kan aantasten.</t>
+          <t>Bij sarcoïdose vormen zich kleine ontstekingshaardjes (granulomen) in uw longen, lymfeklieren of andere organen. De oorzaak is onbekend. Veel patiënten hebben weinig klachten en herstellen spontaan; bij anderen is een behandeling met medicatie nodig.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Herhaaldelijke ademstops tijdens het slapen door obstructie van de bovenste luchtwegen.</t>
+          <t>Bij slaapapneu stopt uw ademhaling herhaaldelijk tijdens de slaap doordat de keel dichtklakt. U slaapt onrustig, snurkt luid en bent overdag vermoeid. Na diagnose via een slaaponderzoek is behandeling met een CPAP-masker of aanpassing van leefstijl zeer doeltreffend.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Littekenvorming in het longweefsel (longfibrose) met progressief verlies van longcapaciteit.</t>
+          <t>Bij interstitiële longziekten ontstaat er littekenweefsel (fibrose) in de longen, waardoor de zuurstofopname verslechtert. U merkt dit aan toenemende kortademigheid en een droge hoest. Vroegtijdige opsporing en behandeling zijn belangrijk om de longfunctie zo lang mogelijk te bewaren.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Vochtophoping of ontsteking in de pleuraholte.</t>
+          <t>Het vlies rond uw longen (het borstvlies) kan ontstoken raken of er kan vocht ophopen. Dit geeft pijn bij het ademhalen en kortademigheid. Via echografie stellen wij de diagnose en kunnen we het vocht zo nodig veilig afvoeren.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Virale en bacteriële infecties van de luchtwegen inclusief influenza en tuberculose.</t>
+          <t>Luchtweginfecties door virussen of bacteriën — van een zware griep tot tuberculose — kunnen de longen ernstig aantasten. Klachten zijn koorts, hoest, kortademigheid en algemene malaise. Wij onderzoeken de oorzaak en starten de gepaste behandeling.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Klinieken-vertalingen compleet + pitch presentatie
</commit_message>
<xml_diff>
--- a/data/aandoeningen.xlsx
+++ b/data/aandoeningen.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -497,6 +497,26 @@
           <t>Volgorde</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Klachten</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Diagnose</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Behandeling</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Wanneer arts</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -527,6 +547,26 @@
       <c r="F2" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Kortademigheid (vooral 's nachts of bij inspanning), piepende ademhaling, beklemmend gevoel op de borst, hoestbuien. Klachten komen vaak in aanvallen en kunnen getriggerd worden door koude lucht, inspanning, pollen of huisstofmijt.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Longfunctiemeting (spirometrie) met reversibiliteitstest, piekstroommeting thuis, eventueel histamine-provocatietest of allergietesten (huidpriktest of bloedonderzoek).</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Inhalatiemedicatie: luchtwegverwijders voor acute klachten, ontstekingsremmers (corticosteroïden) als onderhoudsbehandeling. Bij ernstig astma: biologische therapie. Daarnaast: allergenen vermijden, astma-actieplan opstellen.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Bij aanhoudende hoest of piepen langer dan 3 weken, nachtelijke klachten die uw slaap verstoren, of als uw puffer onvoldoende helpt.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -557,6 +597,26 @@
       <c r="F3" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Niezen, loopneus, jeukende/waterige ogen, huiduitslag, benauwdheid. Bij ernstige allergie: zwelling van de keel, ademhalingsproblemen (anafylaxie — bel 112).</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Huidpriktest (pricktest) met veelvoorkomende allergenen, bloedonderzoek (specifiek IgE), eventueel provocatietest. Resultaat meestal dezelfde dag beschikbaar.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Allergeen vermijden (sanering), antihistaminica, neusspray met corticosteroïden. Bij onvoldoende effect: immunotherapie (desensibilisatie) — een kuur van 3 tot 5 jaar die de allergie aan de bron aanpakt.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Bij terugkerende of erger wordende klachten, onvoldoende effect van vrij verkrijgbare medicatie, of als u wilt weten op welk allergeen u reageert.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -587,6 +647,26 @@
       <c r="F4" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Toenemende kortademigheid (eerst bij inspanning, later ook in rust), chronische hoest met slijm, snelle vermoeidheid, frequente luchtweginfecties. Klachten verergeren vaak in de herfst en winter.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Spirometrie (longfunctietest): als de luchtwegen onvoldoende opengaan na medicatie, wijst dit op COPD. Aanvullend: CT-scan, bloedgasanalyse, inspanningstest (CPET) om de ernst in te schatten.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Rookstop is de belangrijkste stap. Verder: inhalatiemedicatie (luchtwegverwijders + ontstekingsremmers), longrevalidatie, zuurstoftherapie bij ernstige COPD, vaccinatie tegen griep en pneumokokken.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Bij toenemende kortademigheid, hoest langer dan 3 weken, opgeven van bloed of slijm, of als u (ex-)roker bent boven de 40 jaar.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -617,6 +697,26 @@
       <c r="F5" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Koorts (soms met rillingen), hoest met slijm (soms groenig of bloederig), kortademigheid, pijn op de borst bij diep inademen, vermoeidheid en algemeen ziektegevoel.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Klinisch onderzoek (beluisteren van de longen), bloedonderzoek (ontstekingswaarden), thoraxfoto (RX), eventueel CT-scan of sputumkweek om de verwekker te identificeren.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Antibiotica bij bacteriële pneumonie, rust en vochtinname. Bij ernstige gevallen: ziekenhuisopname met intraveneuze antibiotica en zuurstof. Virale pneumonieën genezen meestal met ondersteunende zorg.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Bij koorts boven 38,5°C met hoest en kortademigheid, pijn op de borst, of als klachten na een week niet verbeteren.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -647,6 +747,26 @@
       <c r="F6" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Plotse, stekende pijn op de borst (aan één zijde), kortademigheid die snel verergert, soms droge hoest. Ontstaat spontaan (vooral bij jonge, slanke mannen) of na een trauma.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Thoraxfoto (RX) of CT-scan toont de ingeklapte long. Bij spoed kan echografie aan het bed een snelle diagnose geven.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Kleine klaplong: observatie en rust. Grotere klaplong: afzuigen van lucht via een naald of drainbuis. Bij terugkerende klaplong: chirurgische ingreep (pleurodese of thoracoscopie).</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Bij plotse eenzijdige borstpijn met ademhalingsproblemen: ga onmiddellijk naar de spoedafdeling.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -677,6 +797,26 @@
       <c r="F7" s="2" t="n">
         <v>6</v>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Plotse kortademigheid, stekende pijn op de borst (erger bij diep inademen), versnelde hartslag, soms bloed ophoesten, lichthoofdigheid. Risicofactoren: recente operatie, lange immobilisatie, anticonceptiepil, trombose in het verleden.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>D-dimeer-bloedtest (bij lage verdenking), CT-angiografie van de longen (gouden standaard). Soms aanvullend: echografie van de benen om diepe veneuze trombose op te sporen.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Bloedverdunners (anticoagulantia) gedurende minstens 3 maanden. Bij massale embolie: trombolyse of katheteringreep. Daarna: opvolging en eventueel langdurige bloedverdunning.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Bij plotse kortademigheid met borstpijn: bel 112. Dit is een spoedgeval.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -707,6 +847,26 @@
       <c r="F8" s="2" t="n">
         <v>7</v>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Aanhoudende hoest (of verandering van een bestaande hoest), bloed ophoesten, onverklaard gewichtsverlies, aanhoudende moeheid, pijn op de borst, terugkerende longinfecties. In een vroeg stadium zijn er vaak geen klachten.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>CT-scan van de longen, PET-scan, bronchoscopie met biopsie, EBUS (echo-endoscopie) voor lymfeklieronderzoek. Elke patiënt wordt besproken in het wekelijks multidisciplinair overleg (MOC).</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Afhankelijk van het stadium: chirurgie, chemotherapie, immunotherapie, bestraling, of een combinatie. Het behandelplan wordt op maat gemaakt door het MOC-team (longarts, chirurg, oncoloog, radioloog, patholoog).</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Bij aanhoudende hoest langer dan 3 weken, bloed ophoesten, onverklaard gewichtsverlies, of als u (ex-)roker bent en zich zorgen maakt.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -737,6 +897,26 @@
       <c r="F9" s="2" t="n">
         <v>8</v>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Vaak weinig klachten bij ontdekking. Mogelijke symptomen: droge hoest, moeheid, kortademigheid bij inspanning, gewrichtspijn, huidafwijkingen, koorts. De ziekte kan ook ogen, lever en hart treffen.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Thoraxfoto en CT-scan (vergrote lymfeklieren, longafwijkingen), bloedonderzoek (ACE-spiegel, calcium), longfunctietest. Soms weefselbiopsie via bronchoscopie ter bevestiging.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Bij milde vormen: afwachtend beleid met regelmatige controles. Bij ernstigere vormen: corticosteroïden (prednison), soms aangevuld met methotrexaat of andere immuunonderdrukkende medicatie.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Bij onverklaarde moeheid gecombineerd met hoest of kortademigheid, of bij huidafwijkingen die niet verdwijnen.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -767,6 +947,26 @@
       <c r="F10" s="2" t="n">
         <v>9</v>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Luid snurken, ademstops opgemerkt door partner, onrustige slaap, overmatige slaperigheid overdag, concentratieproblemen, ochtendhoofpijn, prikkelbaarheid. Verhoogt risico op hoge bloeddruk en hart- en vaatziekten.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Polysomnografie (uitgebreide slaapstudie in het slaaplabo): we meten ademhaling, zuurstof, hersenactiviteit, hartritme en spierbewegingen tijdens uw slaap. Soms eerst een screeningstest thuis.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>CPAP-therapie (masker dat uw luchtwegen openhoudt tijdens de slaap) is de standaardbehandeling. Daarnaast: gewichtsreductie, zijligging, vermijden van alcohol voor het slapengaan. Bij mildere vormen: gebitsprothese (MRA).</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Bij dagelijkse vermoeidheid ondanks voldoende slaap, luid snurken met ademstops, of als uw partner zich zorgen maakt over uw ademhaling 's nachts.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -797,6 +997,26 @@
       <c r="F11" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Geleidelijk toenemende kortademigheid (eerst bij inspanning, later ook in rust), droge prikkelhoest, vermoeidheid. Soms knettergeluiden hoorbaar met de stethoscoop ('velcro-crackles') en trommelstokvingers.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>HRCT-scan (hoge-resolutie CT) toont het patroon van fibrose, longfunctietest met diffusiemeting (DLCO), bloedonderzoek op auto-immuunziekten, soms longbiopsie via thoracoscopie.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Antifibrotische medicatie (pirfenidon of nintedanib) vertraagt de achteruitgang bij longfibrose (IPF). Bij andere vormen: immuunonderdrukkende therapie. Zuurstoftherapie en longrevalidatie verbeteren de levenskwaliteit. In uitzonderlijke gevallen: longtransplantatie.</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Bij onverklaarde kortademigheid die langzaam verergert, droge hoest langer dan 8 weken, of als u een auto-immuunziekte heeft en longklachten ontwikkelt.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -827,6 +1047,26 @@
       <c r="F12" s="2" t="n">
         <v>11</v>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Scherpe, stekende pijn op de borst die verergert bij diep inademen of hoesten (pleuritis), kortademigheid bij vochtophoping (pleuravocht). Soms koorts bij infectie.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Echografie van de thorax (snel en pijnloos), thoraxfoto, CT-scan. Bij pleuravocht: punctie (pleurapunctie) voor analyse van het vocht om de oorzaak te achterhalen.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Behandeling van de onderliggende oorzaak (infectie, hartfalen, kanker). Bij veel vocht: afvoeren via punctie of drain. Bij terugkerend vocht: pleurodese (verkleven van de longvliezen) of tunneldrain voor thuisgebruik.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Bij pijn op de borst bij het ademhalen, toenemende kortademigheid, of koorts met borstpijn.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -856,6 +1096,26 @@
       </c>
       <c r="F13" s="2" t="n">
         <v>12</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Koorts, hoest, keelpijn, spierpijn, vermoeidheid, hoofdpijn. Bij ernstige infecties: hoge koorts, kortademigheid, verwardheid. Risicopatiënten: ouderen, zwangeren, mensen met hart- of longziekten.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Klinisch onderzoek, eventueel neusswab (PCR-test voor influenza/COVID/RSV), thoraxfoto bij vermoeden van longontsteking, bloedonderzoek.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Rust, vochtinname, koortsverlaging. Bij griep kan antivirale medicatie (oseltamivir) helpen als deze vroeg wordt gestart. Preventie: jaarlijkse griepvaccinatie, COVID-vaccinatie, handhygiëne.</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Bij koorts langer dan 5 dagen, ernstige kortademigheid, pijn op de borst, of als u tot een risicogroep behoort.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>